<commit_message>
feat: update service fee structure — $6,500 setup, 15% mgmt fee on ad + influencer spend
- Setup fee: $5,000 → $6,500 (one-time Month 1)
- Add 15% management fee on Meta Ads + influencer spend from Month 2
- Jenny's total Year 1: $78,200 → $92,814
- Grand total budget: $174,025 → $188,639
- Update Excel, EN deck, and ZH deck

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KKlue_Year1_Budget.xlsx
+++ b/KKlue_Year1_Budget.xlsx
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="57" min="1" max="1"/>
@@ -942,10 +942,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="16" t="n">
-        <v>11100</v>
+        <v>12600</v>
       </c>
       <c r="J6" s="17" t="n">
-        <v>11800</v>
+        <v>13300</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" s="57">
@@ -978,10 +978,10 @@
         <v>0</v>
       </c>
       <c r="I7" s="16" t="n">
-        <v>6100</v>
+        <v>6846</v>
       </c>
       <c r="J7" s="17" t="n">
-        <v>11775</v>
+        <v>12521</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" s="57">
@@ -1014,10 +1014,10 @@
         <v>0</v>
       </c>
       <c r="I8" s="16" t="n">
-        <v>6100</v>
+        <v>6989</v>
       </c>
       <c r="J8" s="17" t="n">
-        <v>12725</v>
+        <v>13614</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" s="57">
@@ -1050,10 +1050,10 @@
         <v>0</v>
       </c>
       <c r="I9" s="16" t="n">
-        <v>6100</v>
+        <v>6835</v>
       </c>
       <c r="J9" s="17" t="n">
-        <v>11700</v>
+        <v>12435</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" s="57">
@@ -1086,10 +1086,10 @@
         <v>0</v>
       </c>
       <c r="I10" s="16" t="n">
-        <v>6100</v>
+        <v>6985</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>12700</v>
+        <v>13585</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" s="57">
@@ -1122,10 +1122,10 @@
         <v>0</v>
       </c>
       <c r="I11" s="16" t="n">
-        <v>6100</v>
+        <v>7356</v>
       </c>
       <c r="J11" s="17" t="n">
-        <v>15175</v>
+        <v>16431</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" s="57">
@@ -1158,10 +1158,10 @@
         <v>0</v>
       </c>
       <c r="I12" s="16" t="n">
-        <v>6100</v>
+        <v>7675</v>
       </c>
       <c r="J12" s="17" t="n">
-        <v>17300</v>
+        <v>18875</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" s="57">
@@ -1194,10 +1194,10 @@
         <v>0</v>
       </c>
       <c r="I13" s="16" t="n">
-        <v>6100</v>
+        <v>7979</v>
       </c>
       <c r="J13" s="17" t="n">
-        <v>19325</v>
+        <v>21204</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" s="57">
@@ -1230,10 +1230,10 @@
         <v>0</v>
       </c>
       <c r="I14" s="16" t="n">
-        <v>6100</v>
+        <v>8125</v>
       </c>
       <c r="J14" s="17" t="n">
-        <v>20300</v>
+        <v>22325</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" s="57">
@@ -1266,10 +1266,10 @@
         <v>0</v>
       </c>
       <c r="I15" s="16" t="n">
-        <v>6100</v>
+        <v>7300</v>
       </c>
       <c r="J15" s="17" t="n">
-        <v>14800</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" s="57">
@@ -1302,10 +1302,10 @@
         <v>0</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>6100</v>
+        <v>7300</v>
       </c>
       <c r="J16" s="17" t="n">
-        <v>14800</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" s="57">
@@ -1338,10 +1338,10 @@
         <v>0</v>
       </c>
       <c r="I17" s="16" t="n">
-        <v>6100</v>
+        <v>6824</v>
       </c>
       <c r="J17" s="17" t="n">
-        <v>11625</v>
+        <v>12349</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" s="57">
@@ -1391,7 +1391,7 @@
     <row r="21" ht="14" customHeight="1" s="57">
       <c r="A21" s="58" t="inlineStr">
         <is>
-          <t>Month 1 Jenny fee = Phase 0 one-time $5,000 + Month 1 retainer $6,100 = $11,100</t>
+          <t>Month 1 Jenny fee = Phase 0 one-time $6,500 + Month 1 retainer $6,100 = $12,600</t>
         </is>
       </c>
     </row>
@@ -1425,6 +1425,13 @@
     </row>
     <row r="26" ht="14" customHeight="1" s="57">
       <c r="A26" s="58" t="inlineStr">
+        <is>
+          <t>15% management fee applied on Meta Ads + Influencer spend from Month 2 onward</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Etsy = minimal test in Month 2 to measure US search intent for fine jewelry keywords</t>
         </is>
@@ -1477,7 +1484,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="22" customHeight="1" s="57">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -1510,7 +1516,7 @@
         <v>59400</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>0.3407556385576785</v>
+        <v>0.3148871654323867</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
@@ -1525,14 +1531,14 @@
         </is>
       </c>
       <c r="B6" s="28" t="n">
-        <v>78200</v>
+        <v>92814</v>
       </c>
       <c r="C6" s="29" t="n">
-        <v>0.4493607240339031</v>
+        <v>0.492019147684201</v>
       </c>
       <c r="D6" s="30" t="inlineStr">
         <is>
-          <t>Phase 0 $5,000 + $6,100/mo × 12 months</t>
+          <t>Phase 0 $6,500 + $6,100/mo × 12 months + 15% mgmt fee on Meta Ads + Influencer spend</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1552,7 @@
         <v>16625</v>
       </c>
       <c r="C7" s="33" t="n">
-        <v>0.09553225111334579</v>
+        <v>0.08813129840594999</v>
       </c>
       <c r="D7" s="34" t="inlineStr">
         <is>
@@ -1564,7 +1570,7 @@
         <v>11400</v>
       </c>
       <c r="C8" s="33" t="n">
-        <v>0.06550782933486568</v>
+        <v>0.06043289033550856</v>
       </c>
       <c r="D8" s="34" t="inlineStr">
         <is>
@@ -1600,7 +1606,7 @@
         <v>8400</v>
       </c>
       <c r="C10" s="37" t="n">
-        <v>0.0482689269</v>
+        <v>0.04452949814195368</v>
       </c>
       <c r="D10" s="38" t="inlineStr">
         <is>
@@ -1633,14 +1639,13 @@
         </is>
       </c>
       <c r="B12" s="44" t="n">
-        <v>174025</v>
+        <v>188639</v>
       </c>
       <c r="C12" s="45" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="46" t="n"/>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
@@ -1668,7 +1673,7 @@
       </c>
       <c r="B16" s="48" t="inlineStr">
         <is>
-          <t>$174,025</t>
+          <t>$188,639</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1685,7 @@
       </c>
       <c r="B17" s="48" t="inlineStr">
         <is>
-          <t>99% of $175K midpoint</t>
+          <t>107.8% of $175K midpoint</t>
         </is>
       </c>
     </row>

</xml_diff>